<commit_message>
Commit Updating Workbook on 13-08-2026
</commit_message>
<xml_diff>
--- a/12600351.xlsx
+++ b/12600351.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sage/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EA6FDF2-6696-AB47-8B30-4EF324CFACEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2567E296-0D84-2A43-A1BD-8284B050907B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17200" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="59">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -206,6 +206,15 @@
   <si>
     <t>August</t>
   </si>
+  <si>
+    <t>Unsatisfied</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>A divinely boring day overall. 7 out of 8 lectures were boring, making the day feel endless.</t>
+  </si>
 </sst>
 </file>
 
@@ -227,73 +236,73 @@
       <sz val="18"/>
       <color rgb="FF1F4E78"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="13"/>
       <color rgb="FF595959"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <color rgb="FF595959"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10.5"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF1F4E78"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="13"/>
       <color rgb="FF1F4E78"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF595959"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF808080"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -875,7 +884,7 @@
   <dimension ref="A1:N401"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" customWidth="1"/>
+    <col min="1" max="1" width="33.33203125" customWidth="1"/>
     <col min="2" max="4" width="11" customWidth="1"/>
     <col min="5" max="5" width="23" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
@@ -1048,27 +1057,51 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A7" s="12"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="14" t="str">
+    <row r="7" spans="1:14" ht="48" x14ac:dyDescent="0.2">
+      <c r="A7" s="12">
+        <v>46247</v>
+      </c>
+      <c r="B7" s="13">
+        <v>460</v>
+      </c>
+      <c r="C7" s="13">
+        <v>0</v>
+      </c>
+      <c r="D7" s="13">
+        <v>60</v>
+      </c>
+      <c r="E7" s="13">
+        <v>60</v>
+      </c>
+      <c r="F7" s="13">
+        <v>400</v>
+      </c>
+      <c r="G7" s="13">
+        <v>8</v>
+      </c>
+      <c r="H7" s="13">
+        <v>120</v>
+      </c>
+      <c r="I7" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J7" s="14" t="str">
+        <v>1100</v>
+      </c>
+      <c r="J7" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K7" s="15"/>
-      <c r="L7" s="15"/>
-      <c r="M7" s="15"/>
-      <c r="N7" s="16"/>
+        <v>340</v>
+      </c>
+      <c r="K7" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="L7" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="M7" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="N7" s="16" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" s="12"/>

</xml_diff>

<commit_message>
Commit for 14 Aug 2026
</commit_message>
<xml_diff>
--- a/12600351.xlsx
+++ b/12600351.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sage/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2567E296-0D84-2A43-A1BD-8284B050907B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{465A96BE-6573-A340-8B5B-C4293B43C568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17200" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="63">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -215,6 +215,18 @@
   <si>
     <t>A divinely boring day overall. 7 out of 8 lectures were boring, making the day feel endless.</t>
   </si>
+  <si>
+    <t>Excellent</t>
+  </si>
+  <si>
+    <t>Satisfied</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Today was a genuinely nice day. The lectures felt engaging, the atmosphere was pleasant, and overall the day passed by smoothly. After yesterday’s endless lectures, today was a refreshing change and left me in a much better mood.</t>
+  </si>
 </sst>
 </file>
 
@@ -223,7 +235,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -318,6 +330,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -366,7 +384,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -413,6 +431,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1099,31 +1120,55 @@
       <c r="M7" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="N7" s="16" t="s">
+      <c r="N7" s="22" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A8" s="12"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="14" t="str">
+    <row r="8" spans="1:14" ht="128" x14ac:dyDescent="0.2">
+      <c r="A8" s="12">
+        <v>46248</v>
+      </c>
+      <c r="B8" s="13">
+        <v>300</v>
+      </c>
+      <c r="C8" s="13">
+        <v>0</v>
+      </c>
+      <c r="D8" s="13">
+        <v>120</v>
+      </c>
+      <c r="E8" s="13">
+        <v>60</v>
+      </c>
+      <c r="F8" s="13">
+        <v>350</v>
+      </c>
+      <c r="G8" s="13">
+        <v>7</v>
+      </c>
+      <c r="H8" s="13">
+        <v>300</v>
+      </c>
+      <c r="I8" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J8" s="14" t="str">
+        <v>1130</v>
+      </c>
+      <c r="J8" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K8" s="15"/>
-      <c r="L8" s="15"/>
-      <c r="M8" s="15"/>
-      <c r="N8" s="16"/>
+        <v>310</v>
+      </c>
+      <c r="K8" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="L8" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="M8" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="N8" s="16" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="12"/>

</xml_diff>

<commit_message>
Commit for 15 Aug
</commit_message>
<xml_diff>
--- a/12600351.xlsx
+++ b/12600351.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sage/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{465A96BE-6573-A340-8B5B-C4293B43C568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{704DEF51-4129-9442-AF3B-0A8EC416B2EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17200" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="65">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -226,6 +226,12 @@
   </si>
   <si>
     <t>Today was a genuinely nice day. The lectures felt engaging, the atmosphere was pleasant, and overall the day passed by smoothly. After yesterday’s endless lectures, today was a refreshing change and left me in a much better mood.</t>
+  </si>
+  <si>
+    <t>Very Satisfied</t>
+  </si>
+  <si>
+    <t>Went along with my friends to wagha border so see parade on independence day.</t>
   </si>
 </sst>
 </file>
@@ -428,12 +434,12 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -919,74 +925,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
     </row>
     <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
       <c r="E2" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="21">
+      <c r="F2" s="22">
         <v>12600351</v>
       </c>
-      <c r="G2" s="21"/>
+      <c r="G2" s="22"/>
     </row>
     <row r="3" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
       <c r="E3" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="21" t="s">
+      <c r="F3" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="G3" s="21"/>
+      <c r="G3" s="22"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+      <c r="M4" s="20"/>
+      <c r="N4" s="20"/>
     </row>
     <row r="5" spans="1:14" ht="45" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
@@ -1120,7 +1126,7 @@
       <c r="M7" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="N7" s="22" t="s">
+      <c r="N7" s="19" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1170,27 +1176,51 @@
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A9" s="12"/>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="14" t="str">
+    <row r="9" spans="1:14" ht="48" x14ac:dyDescent="0.2">
+      <c r="A9" s="12">
+        <v>46249</v>
+      </c>
+      <c r="B9" s="13">
+        <v>480</v>
+      </c>
+      <c r="C9" s="13">
+        <v>0</v>
+      </c>
+      <c r="D9" s="13">
+        <v>0</v>
+      </c>
+      <c r="E9" s="13">
+        <v>0</v>
+      </c>
+      <c r="F9" s="13">
+        <v>0</v>
+      </c>
+      <c r="G9" s="13">
+        <v>0</v>
+      </c>
+      <c r="H9" s="13">
+        <v>900</v>
+      </c>
+      <c r="I9" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J9" s="14" t="str">
+        <v>1380</v>
+      </c>
+      <c r="J9" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K9" s="15"/>
-      <c r="L9" s="15"/>
-      <c r="M9" s="15"/>
-      <c r="N9" s="16"/>
+        <v>60</v>
+      </c>
+      <c r="K9" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="L9" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="M9" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="N9" s="16" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" s="12"/>

</xml_diff>

<commit_message>
Commit for 16 Aug 2026
</commit_message>
<xml_diff>
--- a/12600351.xlsx
+++ b/12600351.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sage/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{704DEF51-4129-9442-AF3B-0A8EC416B2EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DF1EA47-25B9-5046-AE55-4828283DCE8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17200" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="67">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -232,6 +232,12 @@
   </si>
   <si>
     <t>Went along with my friends to wagha border so see parade on independence day.</t>
+  </si>
+  <si>
+    <t>156/08/2026</t>
+  </si>
+  <si>
+    <t>Did some DSA, and worked on a npm package.</t>
   </si>
 </sst>
 </file>
@@ -1222,27 +1228,51 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A10" s="12"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="14" t="str">
+    <row r="10" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+      <c r="A10" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" s="13">
+        <v>480</v>
+      </c>
+      <c r="C10" s="13">
+        <v>0</v>
+      </c>
+      <c r="D10" s="13">
+        <v>0</v>
+      </c>
+      <c r="E10" s="13">
+        <v>180</v>
+      </c>
+      <c r="F10" s="13">
+        <v>0</v>
+      </c>
+      <c r="G10" s="13">
+        <v>0</v>
+      </c>
+      <c r="H10" s="13">
+        <v>600</v>
+      </c>
+      <c r="I10" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J10" s="14" t="str">
+        <v>1260</v>
+      </c>
+      <c r="J10" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K10" s="15"/>
-      <c r="L10" s="15"/>
-      <c r="M10" s="15"/>
-      <c r="N10" s="16"/>
+        <v>180</v>
+      </c>
+      <c r="K10" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="L10" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="M10" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="N10" s="16" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" s="12"/>

</xml_diff>

<commit_message>
Commit for 17 Aug 2026
</commit_message>
<xml_diff>
--- a/12600351.xlsx
+++ b/12600351.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sage/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DF1EA47-25B9-5046-AE55-4828283DCE8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCC97C33-19EF-D74E-84A5-5E806135972D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17200" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="67">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -234,10 +234,10 @@
     <t>Went along with my friends to wagha border so see parade on independence day.</t>
   </si>
   <si>
-    <t>156/08/2026</t>
+    <t>Did some DSA, and worked on a npm package.</t>
   </si>
   <si>
-    <t>Did some DSA, and worked on a npm package.</t>
+    <t>Did some DSA.</t>
   </si>
 </sst>
 </file>
@@ -1229,8 +1229,8 @@
       </c>
     </row>
     <row r="10" spans="1:14" ht="32" x14ac:dyDescent="0.2">
-      <c r="A10" s="12" t="s">
-        <v>65</v>
+      <c r="A10" s="12">
+        <v>46250</v>
       </c>
       <c r="B10" s="13">
         <v>480</v>
@@ -1271,30 +1271,54 @@
         <v>57</v>
       </c>
       <c r="N10" s="16" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="12">
+        <v>46251</v>
+      </c>
+      <c r="B11" s="13">
+        <v>480</v>
+      </c>
+      <c r="C11" s="13">
+        <v>0</v>
+      </c>
+      <c r="D11" s="13">
+        <v>0</v>
+      </c>
+      <c r="E11" s="13">
+        <v>180</v>
+      </c>
+      <c r="F11" s="13">
+        <v>0</v>
+      </c>
+      <c r="G11" s="13">
+        <v>0</v>
+      </c>
+      <c r="H11" s="13">
+        <v>600</v>
+      </c>
+      <c r="I11" s="14">
+        <f t="shared" si="0"/>
+        <v>1260</v>
+      </c>
+      <c r="J11" s="14">
+        <f t="shared" si="1"/>
+        <v>180</v>
+      </c>
+      <c r="K11" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="L11" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="M11" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="N11" s="16" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A11" s="12"/>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="14" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J11" s="14" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K11" s="15"/>
-      <c r="L11" s="15"/>
-      <c r="M11" s="15"/>
-      <c r="N11" s="16"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" s="12"/>

</xml_diff>

<commit_message>
Commit for 28 Aug 1016
</commit_message>
<xml_diff>
--- a/12600351.xlsx
+++ b/12600351.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sage/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8D9E7A0-F7C1-AB4A-A10E-AA7E24B54F3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ADD9C12-8C52-9842-8692-DCF8D17B6005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17200" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="79">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -271,6 +271,9 @@
   </si>
   <si>
     <t>Did DSA problems, average day.</t>
+  </si>
+  <si>
+    <t>RakshaBandhan</t>
   </si>
 </sst>
 </file>
@@ -1725,7 +1728,9 @@
       <c r="A20" s="12">
         <v>46260</v>
       </c>
-      <c r="B20" s="13"/>
+      <c r="B20" s="13">
+        <v>480</v>
+      </c>
       <c r="C20" s="13">
         <v>0</v>
       </c>
@@ -1746,11 +1751,11 @@
       </c>
       <c r="I20" s="14">
         <f t="shared" si="0"/>
-        <v>920</v>
+        <v>1400</v>
       </c>
       <c r="J20" s="14">
         <f t="shared" si="1"/>
-        <v>520</v>
+        <v>40</v>
       </c>
       <c r="K20" s="15" t="s">
         <v>52</v>
@@ -1769,7 +1774,9 @@
       <c r="A21" s="12">
         <v>46261</v>
       </c>
-      <c r="B21" s="13"/>
+      <c r="B21" s="13">
+        <v>480</v>
+      </c>
       <c r="C21" s="13">
         <v>0</v>
       </c>
@@ -1786,15 +1793,15 @@
         <v>7</v>
       </c>
       <c r="H21" s="13">
-        <v>450</v>
+        <v>200</v>
       </c>
       <c r="I21" s="14">
         <f t="shared" si="0"/>
-        <v>1160</v>
+        <v>1390</v>
       </c>
       <c r="J21" s="14">
         <f t="shared" si="1"/>
-        <v>280</v>
+        <v>50</v>
       </c>
       <c r="K21" s="15" t="s">
         <v>59</v>
@@ -1809,27 +1816,51 @@
         <v>77</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A22" s="12"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="13"/>
-      <c r="H22" s="13"/>
-      <c r="I22" s="14" t="str">
+    <row r="22" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+      <c r="A22" s="12">
+        <v>46262</v>
+      </c>
+      <c r="B22" s="13">
+        <v>480</v>
+      </c>
+      <c r="C22" s="13">
+        <v>0</v>
+      </c>
+      <c r="D22" s="13">
+        <v>0</v>
+      </c>
+      <c r="E22" s="13">
+        <v>250</v>
+      </c>
+      <c r="F22" s="13">
+        <v>0</v>
+      </c>
+      <c r="G22" s="13">
+        <v>0</v>
+      </c>
+      <c r="H22" s="13">
+        <v>700</v>
+      </c>
+      <c r="I22" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="14" t="str">
+        <v>1430</v>
+      </c>
+      <c r="J22" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="15"/>
-      <c r="L22" s="15"/>
-      <c r="M22" s="15"/>
-      <c r="N22" s="16"/>
+        <v>10</v>
+      </c>
+      <c r="K22" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="L22" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="M22" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="N22" s="16" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A23" s="12"/>

</xml_diff>

<commit_message>
Commit for 1st September 2026
</commit_message>
<xml_diff>
--- a/12600351.xlsx
+++ b/12600351.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sage/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9A083F6-D248-E043-B38D-1D87EE1B4B5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{858844DE-98B6-E04C-9630-98A89DF1C7F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17200" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="81">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -277,6 +277,9 @@
   </si>
   <si>
     <t>Learned Complete SQL for RPL exam.</t>
+  </si>
+  <si>
+    <t>Started Solving Frontend Problems asked by FANG Companies.</t>
   </si>
 </sst>
 </file>
@@ -2003,27 +2006,51 @@
         <v>79</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A26" s="12"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="13"/>
-      <c r="H26" s="13"/>
-      <c r="I26" s="14" t="str">
+    <row r="26" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+      <c r="A26" s="12">
+        <v>46266</v>
+      </c>
+      <c r="B26" s="13">
+        <v>390</v>
+      </c>
+      <c r="C26" s="13">
+        <v>0</v>
+      </c>
+      <c r="D26" s="13">
+        <v>150</v>
+      </c>
+      <c r="E26" s="13">
+        <v>370</v>
+      </c>
+      <c r="F26" s="13">
+        <v>350</v>
+      </c>
+      <c r="G26" s="13">
+        <v>7</v>
+      </c>
+      <c r="H26" s="13">
+        <v>100</v>
+      </c>
+      <c r="I26" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J26" s="14" t="str">
+        <v>1360</v>
+      </c>
+      <c r="J26" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K26" s="15"/>
-      <c r="L26" s="15"/>
-      <c r="M26" s="15"/>
-      <c r="N26" s="16"/>
+        <v>80</v>
+      </c>
+      <c r="K26" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="L26" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="M26" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="N26" s="16" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27" s="12"/>

</xml_diff>